<commit_message>
Site: clear every audit item that did not need an outside fact
- Offerings: "2x faster to first shot" loses the multiple; MIL-STD claim
  scoped to programmes that specify it; "the date is the contract"
  becomes "we hold ourselves to the committed date"
- Case studies: headline "Proof, not promises" becomes "Programmes we
  have delivered"
- BNC case: the unsourced $10M+ benchmark and the "~90% cost" delta are
  gone site-wide, on the index, the chart and the case page. Our own
  under $1M figure stays
- Coffee case: the customer-supplied cost benchmark is withheld pending
  written consent; our own ~$100k stays
- Stock imagery replaced with our own: the LMM Stack factory and
  dashboard shots, and the robot arm on About

Workbook: 27 fixed on branch, 5 partly, 11 not started, 1 drafted. What
is left needs a fact or a decision, not an edit.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_s4/NEMI_website_update_list.xlsx
+++ b/_s4/NEMI_website_update_list.xlsx
@@ -1176,12 +1176,16 @@
           <t>CFO</t>
         </is>
       </c>
-      <c r="J15" s="8" t="inlineStr">
-        <is>
-          <t>Not fixed</t>
-        </is>
-      </c>
-      <c r="K15" s="7" t="inlineStr"/>
+      <c r="J15" s="6" t="inlineStr">
+        <is>
+          <t>Fixed on branch</t>
+        </is>
+      </c>
+      <c r="K15" s="7" t="inlineStr">
+        <is>
+          <t>The unsourced $10M+ benchmark and the 90% delta are gone site-wide. Our own &lt;$1M stays. The site-versus-deck reconciliation is still open.</t>
+        </is>
+      </c>
       <c r="L15" s="7" t="inlineStr"/>
     </row>
     <row r="16">
@@ -1280,12 +1284,16 @@
           <t>Sales + CFO</t>
         </is>
       </c>
-      <c r="J17" s="8" t="inlineStr">
-        <is>
-          <t>Not fixed</t>
-        </is>
-      </c>
-      <c r="K17" s="7" t="inlineStr"/>
+      <c r="J17" s="9" t="inlineStr">
+        <is>
+          <t>Partly fixed</t>
+        </is>
+      </c>
+      <c r="K17" s="7" t="inlineStr">
+        <is>
+          <t>Customer-supplied cost benchmark withheld pending written consent. Our own ~$100k and the delivery facts stay.</t>
+        </is>
+      </c>
       <c r="L17" s="7" t="inlineStr"/>
     </row>
     <row r="18">
@@ -2080,12 +2088,16 @@
           <t>Marketing</t>
         </is>
       </c>
-      <c r="J32" s="8" t="inlineStr">
-        <is>
-          <t>Not fixed</t>
-        </is>
-      </c>
-      <c r="K32" s="7" t="inlineStr"/>
+      <c r="J32" s="6" t="inlineStr">
+        <is>
+          <t>Fixed on branch</t>
+        </is>
+      </c>
+      <c r="K32" s="7" t="inlineStr">
+        <is>
+          <t>Swapped for care-robotics.jpg, our own robotics cell.</t>
+        </is>
+      </c>
       <c r="L32" s="7" t="inlineStr"/>
     </row>
     <row r="33">
@@ -2296,12 +2308,16 @@
           <t>Marketing</t>
         </is>
       </c>
-      <c r="J36" s="8" t="inlineStr">
-        <is>
-          <t>Not fixed</t>
-        </is>
-      </c>
-      <c r="K36" s="7" t="inlineStr"/>
+      <c r="J36" s="6" t="inlineStr">
+        <is>
+          <t>Fixed on branch</t>
+        </is>
+      </c>
+      <c r="K36" s="7" t="inlineStr">
+        <is>
+          <t>Headline is now 'Programmes we have delivered'; kicker matches.</t>
+        </is>
+      </c>
       <c r="L36" s="7" t="inlineStr"/>
     </row>
     <row r="37">
@@ -2564,12 +2580,16 @@
           <t>Marketing</t>
         </is>
       </c>
-      <c r="J41" s="8" t="inlineStr">
-        <is>
-          <t>Not fixed</t>
-        </is>
-      </c>
-      <c r="K41" s="7" t="inlineStr"/>
+      <c r="J41" s="6" t="inlineStr">
+        <is>
+          <t>Fixed on branch</t>
+        </is>
+      </c>
+      <c r="K41" s="7" t="inlineStr">
+        <is>
+          <t>Swapped for our own: fac-assembly.jpg and care-floor-cad.jpg.</t>
+        </is>
+      </c>
       <c r="L41" s="7" t="inlineStr"/>
     </row>
     <row r="42">
@@ -2672,12 +2692,16 @@
           <t>Counsel</t>
         </is>
       </c>
-      <c r="J43" s="8" t="inlineStr">
-        <is>
-          <t>Not fixed</t>
-        </is>
-      </c>
-      <c r="K43" s="7" t="inlineStr"/>
+      <c r="J43" s="6" t="inlineStr">
+        <is>
+          <t>Fixed on branch</t>
+        </is>
+      </c>
+      <c r="K43" s="7" t="inlineStr">
+        <is>
+          <t>Now 'we hold ourselves to the committed date'. No longer phrased as a contract term.</t>
+        </is>
+      </c>
       <c r="L43" s="7" t="inlineStr"/>
     </row>
     <row r="44">
@@ -2724,12 +2748,16 @@
           <t>COO</t>
         </is>
       </c>
-      <c r="J44" s="8" t="inlineStr">
-        <is>
-          <t>Not fixed</t>
-        </is>
-      </c>
-      <c r="K44" s="7" t="inlineStr"/>
+      <c r="J44" s="6" t="inlineStr">
+        <is>
+          <t>Fixed on branch</t>
+        </is>
+      </c>
+      <c r="K44" s="7" t="inlineStr">
+        <is>
+          <t>Multiple dropped; reads 'faster to first shot' until a benchmark exists.</t>
+        </is>
+      </c>
       <c r="L44" s="7" t="inlineStr"/>
     </row>
     <row r="45">
@@ -2776,12 +2804,16 @@
           <t>Quality</t>
         </is>
       </c>
-      <c r="J45" s="8" t="inlineStr">
-        <is>
-          <t>Not fixed</t>
-        </is>
-      </c>
-      <c r="K45" s="7" t="inlineStr"/>
+      <c r="J45" s="6" t="inlineStr">
+        <is>
+          <t>Fixed on branch</t>
+        </is>
+      </c>
+      <c r="K45" s="7" t="inlineStr">
+        <is>
+          <t>Now 'built to MIL-STD-810 / 461 requirements where a programme calls for them'.</t>
+        </is>
+      </c>
       <c r="L45" s="7" t="inlineStr"/>
     </row>
     <row r="46">

</xml_diff>

<commit_message>
Workbook: reclassify the UAS image row
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_s4/NEMI_website_update_list.xlsx
+++ b/_s4/NEMI_website_update_list.xlsx
@@ -1044,27 +1044,27 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>NEMI carbon-fibre defense UAS photograph</t>
+          <t>Defense UAS hero: an AI-generated illustration, captioned as the delivered airframe</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Customer property</t>
+          <t>Misleading image</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>A defence customer's airframe published without written consent</t>
+          <t>Not customer property after all: the render is ours. But it read as a photograph of delivered hardware</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>Get consent or replace the image</t>
+          <t>Labelled as an illustration on the case page and the index card</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
@@ -1072,12 +1072,16 @@
           <t>CEO</t>
         </is>
       </c>
-      <c r="J13" s="8" t="inlineStr">
-        <is>
-          <t>Not fixed</t>
-        </is>
-      </c>
-      <c r="K13" s="7" t="inlineStr"/>
+      <c r="J13" s="6" t="inlineStr">
+        <is>
+          <t>Fixed on branch</t>
+        </is>
+      </c>
+      <c r="K13" s="7" t="inlineStr">
+        <is>
+          <t>Confirmed with the CEO on 28 Sep 2026 that the image is AI-generated and illustrative.</t>
+        </is>
+      </c>
       <c r="L13" s="7" t="inlineStr"/>
     </row>
     <row r="14">

</xml_diff>

<commit_message>
Workbook: board and leadership row updated
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_s4/NEMI_website_update_list.xlsx
+++ b/_s4/NEMI_website_update_list.xlsx
@@ -732,7 +732,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Vinod Dasari, Ramesh Mangaleswaran, Sampath Ravinarayanan, Naoya Nishimura, Sam Swaminathan</t>
+          <t>Board and leadership structure</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
@@ -747,12 +747,12 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>Titles and roles differ from the deck; the S-4 lists directors exactly, and family relationships must be disclosed</t>
+          <t>The S-4 lists directors and officers exactly. The site now names four directors and seven officers</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>Confirm each seat, title and any family relationship</t>
+          <t>Structure updated 28 Sep. Still to confirm: each director's formal appointment, and any family relationship among directors and officers</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
@@ -760,12 +760,16 @@
           <t>CEO + counsel</t>
         </is>
       </c>
-      <c r="J7" s="8" t="inlineStr">
-        <is>
-          <t>Not fixed</t>
-        </is>
-      </c>
-      <c r="K7" s="7" t="inlineStr"/>
+      <c r="J7" s="9" t="inlineStr">
+        <is>
+          <t>Partly fixed</t>
+        </is>
+      </c>
+      <c r="K7" s="7" t="inlineStr">
+        <is>
+          <t>Board: Anirudh, Sam Swaminathan, Jingjing Kanik (ind.), Manoj Ganesh (ind.). Leadership: 7. Bios from LinkedIn, need sign-off from each person.</t>
+        </is>
+      </c>
       <c r="L7" s="7" t="inlineStr"/>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Master Plan: restore the page exactly as it is on main
Requested: the founder's letter reads word for word as the live site again.
That brings back the original wording this branch had softened: "The only
way", the cellphone line as a belief statement, "MaaS is profitable on its
own", "profitably, today", and drops the forward-looking statements note.
Only the stylesheet version differs from main (189, so the merged CSS loads).

Update list items #4 and #5 now read "Reverted on branch", with a dated note.
About keeps its softened text.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018MafBKjuv7rZ7cieL7GV7x
</commit_message>
<xml_diff>
--- a/_s4/NEMI_website_update_list.xlsx
+++ b/_s4/NEMI_website_update_list.xlsx
@@ -800,10 +800,14 @@
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>Fixed on branch</t>
-        </is>
-      </c>
-      <c r="K8" s="6" t="n"/>
+          <t>Reverted on branch</t>
+        </is>
+      </c>
+      <c r="K8" s="6" t="inlineStr">
+        <is>
+          <t>5 Oct: Master Plan page restored to the live wording on request, so the letter carries this again. About keeps the softened text.</t>
+        </is>
+      </c>
       <c r="L8" s="6" t="n"/>
     </row>
     <row r="9">
@@ -852,10 +856,14 @@
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>Fixed on branch</t>
-        </is>
-      </c>
-      <c r="K9" s="6" t="n"/>
+          <t>Reverted on branch</t>
+        </is>
+      </c>
+      <c r="K9" s="6" t="inlineStr">
+        <is>
+          <t>5 Oct: Master Plan page restored to the live wording on request, so the letter carries this again. About keeps the softened text.</t>
+        </is>
+      </c>
       <c r="L9" s="6" t="n"/>
     </row>
     <row r="10" ht="22.5" customHeight="1">

</xml_diff>